<commit_message>
donwloading file bug fixed, UI elements bugs fixed
</commit_message>
<xml_diff>
--- a/backend/compression_analysis.xlsx
+++ b/backend/compression_analysis.xlsx
@@ -513,11 +513,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -803,6 +803,276 @@
       </c>
       <c r="G10" t="n">
         <v>40.12345679012346</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45777.00839850694</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Monaco editor.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>brotli</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>559</v>
+      </c>
+      <c r="E11" t="n">
+        <v>293</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47.58</v>
+      </c>
+      <c r="G11" t="n">
+        <v>47.58497316636851</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45777.0093062037</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>p.jpg</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>96257</v>
+      </c>
+      <c r="E12" t="n">
+        <v>83010</v>
+      </c>
+      <c r="F12" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="G12" t="n">
+        <v>13.76211600195311</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>45777.01439627315</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tocheckAWS.txt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>brotli</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>324</v>
+      </c>
+      <c r="E13" t="n">
+        <v>194</v>
+      </c>
+      <c r="F13" t="n">
+        <v>40.12</v>
+      </c>
+      <c r="G13" t="n">
+        <v>40.12345679012346</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>45777.01669523148</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sharjil.jpg</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>118410</v>
+      </c>
+      <c r="E14" t="n">
+        <v>117302</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.9357317794105202</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>45778.03233136574</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Monacoeditor.txt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>559</v>
+      </c>
+      <c r="E15" t="n">
+        <v>368</v>
+      </c>
+      <c r="F15" t="n">
+        <v>65.83184257602862</v>
+      </c>
+      <c r="G15" t="n">
+        <v>34.16815742397138</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>45778.03430743056</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Monacoeditor.txt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>559</v>
+      </c>
+      <c r="E16" t="n">
+        <v>368</v>
+      </c>
+      <c r="F16" t="n">
+        <v>65.83184257602862</v>
+      </c>
+      <c r="G16" t="n">
+        <v>34.16815742397138</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45778.03437085648</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>data-compression-technicality.txt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1477</v>
+      </c>
+      <c r="E17" t="n">
+        <v>801</v>
+      </c>
+      <c r="F17" t="n">
+        <v>54.23155044008124</v>
+      </c>
+      <c r="G17" t="n">
+        <v>45.76844955991876</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45778.03447833333</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sharjil.jpg</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>118410</v>
+      </c>
+      <c r="E18" t="n">
+        <v>117302</v>
+      </c>
+      <c r="F18" t="n">
+        <v>99.06426822058948</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.9357317794105202</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45778.0344899537</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>sharjil.jpg</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>118410</v>
+      </c>
+      <c r="E19" t="n">
+        <v>117302</v>
+      </c>
+      <c r="F19" t="n">
+        <v>99.06426822058948</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.9357317794105202</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45778.03455831019</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tocheckAWS.txt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>gzip</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>324</v>
+      </c>
+      <c r="E20" t="n">
+        <v>211</v>
+      </c>
+      <c r="F20" t="n">
+        <v>65.12345679012346</v>
+      </c>
+      <c r="G20" t="n">
+        <v>34.87654320987654</v>
       </c>
     </row>
   </sheetData>
@@ -822,12 +1092,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
@@ -950,43 +1220,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>324</v>
+        <v>371</v>
       </c>
       <c r="D4" t="n">
         <v>324</v>
       </c>
       <c r="E4" t="n">
-        <v>324</v>
+        <v>559</v>
       </c>
       <c r="F4" t="n">
-        <v>194</v>
+        <v>213.8</v>
       </c>
       <c r="G4" t="n">
         <v>194</v>
       </c>
       <c r="H4" t="n">
-        <v>194</v>
+        <v>293</v>
       </c>
       <c r="I4" t="n">
-        <v>40.12</v>
+        <v>41.61</v>
       </c>
       <c r="J4" t="n">
         <v>40.12</v>
       </c>
       <c r="K4" t="n">
-        <v>40.12</v>
+        <v>47.58</v>
       </c>
       <c r="L4" t="n">
-        <v>40.12</v>
+        <v>41.62</v>
       </c>
       <c r="M4" t="n">
         <v>40.12</v>
       </c>
       <c r="N4" t="n">
-        <v>40.12</v>
+        <v>47.58</v>
       </c>
     </row>
     <row r="5">
@@ -996,43 +1266,43 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C5" t="n">
-        <v>324</v>
+        <v>32596.43</v>
       </c>
       <c r="D5" t="n">
         <v>324</v>
       </c>
       <c r="E5" t="n">
-        <v>324</v>
+        <v>118410</v>
       </c>
       <c r="F5" t="n">
-        <v>211</v>
+        <v>31280.71</v>
       </c>
       <c r="G5" t="n">
         <v>211</v>
       </c>
       <c r="H5" t="n">
-        <v>211</v>
+        <v>117302</v>
       </c>
       <c r="I5" t="n">
-        <v>34.88</v>
+        <v>48.08</v>
       </c>
       <c r="J5" t="n">
-        <v>34.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>34.88</v>
+        <v>99.06</v>
       </c>
       <c r="L5" t="n">
-        <v>34.88</v>
+        <v>26.77</v>
       </c>
       <c r="M5" t="n">
-        <v>34.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="N5" t="n">
-        <v>34.88</v>
+        <v>45.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>